<commit_message>
Add four new optimized assets and sync full intake metadata
Optimize TBS and LTE drop files for web delivery, apply the completed intake sheet to the board, and map website content to product filters.
</commit_message>
<xml_diff>
--- a/content/portfolio-intake.xlsx
+++ b/content/portfolio-intake.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="177">
   <si>
     <t>source_file</t>
   </si>
@@ -235,6 +235,12 @@
     <t>public/media/4-b-purchase-poster.webp</t>
   </si>
   <si>
+    <t>Valentine's Promo</t>
+  </si>
+  <si>
+    <t>Occasion-based discount announcement reel proposal</t>
+  </si>
+  <si>
     <t>4.c Purchase</t>
   </si>
   <si>
@@ -244,12 +250,24 @@
     <t>public/media/4-c-purchase-poster.webp</t>
   </si>
   <si>
+    <t>GiF Engagement</t>
+  </si>
+  <si>
+    <t>Facebook post challenge to reveal discount code</t>
+  </si>
+  <si>
     <t>4.d Purchase (1).png</t>
   </si>
   <si>
     <t>public/media/4-d-purchase-1.webp</t>
   </si>
   <si>
+    <t>Giveaway Campaign</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Friendship day campaign announcement mockup </t>
+  </si>
+  <si>
     <t>6. Expand - Mkt Agency</t>
   </si>
   <si>
@@ -259,6 +277,12 @@
     <t>public/media/6-expand-mkt-agency-poster.webp</t>
   </si>
   <si>
+    <t>Testimonial CTA</t>
+  </si>
+  <si>
+    <t>Success story showcase to attract niche bases</t>
+  </si>
+  <si>
     <t>6.a Expand</t>
   </si>
   <si>
@@ -268,6 +292,12 @@
     <t>public/media/6-a-expand-poster.webp</t>
   </si>
   <si>
+    <t>Blind Test</t>
+  </si>
+  <si>
+    <t>New flavor guessing game concept</t>
+  </si>
+  <si>
     <t>6.c Expand</t>
   </si>
   <si>
@@ -277,6 +307,12 @@
     <t>public/media/6-c-expand-poster.webp</t>
   </si>
   <si>
+    <t>Carousel Slider</t>
+  </si>
+  <si>
+    <t>Instagram carousel feature usage for flavor reveal</t>
+  </si>
+  <si>
     <t>AQOHFRn389BHvQxynwDYaKR2q-gJqagkSumkoyjtySC57kwP44lcRxYg8qUOWeYuIXKPrU2JqyeDYMUgElTiqnFhW2zEIGWyew11nYEFMjtwLw.mp4</t>
   </si>
   <si>
@@ -286,24 +322,66 @@
     <t>public/media/asset-18-poster.webp</t>
   </si>
   <si>
+    <t>competition</t>
+  </si>
+  <si>
+    <t>Pathao 10Y Celebration</t>
+  </si>
+  <si>
+    <t>idea</t>
+  </si>
+  <si>
+    <t>OVC to celebrate 10 years of Pathao for admaking competition</t>
+  </si>
+  <si>
+    <t>Competition</t>
+  </si>
+  <si>
     <t>BIDA Post 1.png</t>
   </si>
   <si>
     <t>public/media/bida-post-1.webp</t>
   </si>
   <si>
+    <t>bida-content</t>
+  </si>
+  <si>
+    <t>Thread Post</t>
+  </si>
+  <si>
+    <t>Post on the 'a thread' trend to tackle lowered investment misconception</t>
+  </si>
+  <si>
+    <t>BIDA</t>
+  </si>
+  <si>
     <t>BIDA Post 2.png</t>
   </si>
   <si>
     <t>public/media/bida-post-2.webp</t>
   </si>
   <si>
+    <t>News Post</t>
+  </si>
+  <si>
+    <t>design</t>
+  </si>
+  <si>
+    <t>Photocard of quote to drive traffic to webinar</t>
+  </si>
+  <si>
     <t>BIDA Print.jpg</t>
   </si>
   <si>
     <t>public/media/bida-print.webp</t>
   </si>
   <si>
+    <t>Newspaper Campaign</t>
+  </si>
+  <si>
+    <t>Launch campaign of matchmaking portal on national dailies</t>
+  </si>
+  <si>
     <t>Grand Final ADM 5.mp4</t>
   </si>
   <si>
@@ -313,12 +391,27 @@
     <t>public/media/grand-final-adm-5-poster.webp</t>
   </si>
   <si>
+    <t>NCC Bank Hero OVC</t>
+  </si>
+  <si>
+    <t>idea|shoot</t>
+  </si>
+  <si>
+    <t>OVC to position NCC Bank's offerings for the Gen-Z youth</t>
+  </si>
+  <si>
     <t>Invitation Turkiye.png</t>
   </si>
   <si>
     <t>public/media/invitation-turkiye.webp</t>
   </si>
   <si>
+    <t>Email Invitation Flyer</t>
+  </si>
+  <si>
+    <t>Invitation card for foreign seminar outreach</t>
+  </si>
+  <si>
     <t>LD 1</t>
   </si>
   <si>
@@ -328,12 +421,24 @@
     <t>public/media/ld-1-poster.webp</t>
   </si>
   <si>
+    <t>Product Intro</t>
+  </si>
+  <si>
+    <t>Instagram stitch to piggyback off viral food buzz</t>
+  </si>
+  <si>
     <t>LD 2</t>
   </si>
   <si>
     <t>public/media/ld-2.webp</t>
   </si>
   <si>
+    <t>Product Anatomy</t>
+  </si>
+  <si>
+    <t>4-slide Facebook carousel for close-up of product</t>
+  </si>
+  <si>
     <t>Speech Reel for Turkiye.mp4</t>
   </si>
   <si>
@@ -343,6 +448,12 @@
     <t>public/media/speech-reel-for-turkiye-poster.webp</t>
   </si>
   <si>
+    <t>Short-form Repurpose</t>
+  </si>
+  <si>
+    <t>Long-form content cut to create reels for socials</t>
+  </si>
+  <si>
     <t>Trade Cookies for Chips _ Love Doughs.webm</t>
   </si>
   <si>
@@ -352,13 +463,13 @@
     <t>public/media/trade-cookies-for-chips-love-doughs-poster.webp</t>
   </si>
   <si>
-    <t>WhatsApp Video 2026-02-02 at 12.54.03 PM.mp4</t>
-  </si>
-  <si>
-    <t>public/media/whatsapp-video-2026-02-02-at-12-54-03-pm.mp4</t>
-  </si>
-  <si>
-    <t>public/media/whatsapp-video-2026-02-02-at-12-54-03-pm-poster.webp</t>
+    <t>Campaign Microsite</t>
+  </si>
+  <si>
+    <t>website</t>
+  </si>
+  <si>
+    <t>Landing page walkthrough of a proposed campaign</t>
   </si>
   <si>
     <t>WhatsApp Video 2026-06-24 at 11.46.52 AM.mp4</t>
@@ -370,6 +481,12 @@
     <t>public/media/whatsapp-video-2026-06-24-at-11-46-52-am-poster.webp</t>
   </si>
   <si>
+    <t>Platform Launch</t>
+  </si>
+  <si>
+    <t>Introduction of platform to show what problem it solves</t>
+  </si>
+  <si>
     <t>নারায়ণগঞ্জে তরুণ-তরুণীদের হাতে কার্ডস্টকের রাজ্য _ The Business Standard.mp4</t>
   </si>
   <si>
@@ -377,6 +494,54 @@
   </si>
   <si>
     <t>public/media/the-business-standard-poster.webp</t>
+  </si>
+  <si>
+    <t>tbs-content</t>
+  </si>
+  <si>
+    <t>Product BTS Coverage</t>
+  </si>
+  <si>
+    <t>News coverage of young entrepreneurs</t>
+  </si>
+  <si>
+    <t>The Business Standard</t>
+  </si>
+  <si>
+    <t>TBS Miniature.mp4</t>
+  </si>
+  <si>
+    <t>Product BTS Coverage 2</t>
+  </si>
+  <si>
+    <t>News coverage of unique business</t>
+  </si>
+  <si>
+    <t>marina tbs.png</t>
+  </si>
+  <si>
+    <t>Infographic 1</t>
+  </si>
+  <si>
+    <t>Content series for promo of a contest</t>
+  </si>
+  <si>
+    <t>kashef tbs.png</t>
+  </si>
+  <si>
+    <t>LTE Case.mp4</t>
+  </si>
+  <si>
+    <t>lte-content</t>
+  </si>
+  <si>
+    <t>Commward-winning Campaign</t>
+  </si>
+  <si>
+    <t>Case video for campaign with strategy involvement</t>
+  </si>
+  <si>
+    <t>LTE Advertising</t>
   </si>
 </sst>
 </file>
@@ -753,7 +918,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
@@ -1145,7 +1310,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>71</v>
       </c>
@@ -1158,239 +1323,719 @@
       <c r="D12" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" t="s">
+        <v>18</v>
+      </c>
+      <c r="H12" t="s">
+        <v>19</v>
+      </c>
+      <c r="I12" t="s">
+        <v>75</v>
+      </c>
+      <c r="J12">
+        <v>2026</v>
+      </c>
+      <c r="K12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D13" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" t="s">
+        <v>18</v>
+      </c>
+      <c r="H13" t="s">
+        <v>40</v>
+      </c>
+      <c r="I13" t="s">
+        <v>80</v>
+      </c>
+      <c r="J13">
+        <v>2026</v>
+      </c>
+      <c r="K13" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D14" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E14" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" t="s">
+        <v>83</v>
+      </c>
+      <c r="G14" t="s">
+        <v>31</v>
+      </c>
+      <c r="H14" t="s">
+        <v>32</v>
+      </c>
+      <c r="I14" t="s">
+        <v>84</v>
+      </c>
+      <c r="J14">
+        <v>2026</v>
+      </c>
+      <c r="K14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="B15" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C15" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="D15" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" t="s">
+        <v>88</v>
+      </c>
+      <c r="G15" t="s">
+        <v>18</v>
+      </c>
+      <c r="H15" t="s">
+        <v>19</v>
+      </c>
+      <c r="I15" t="s">
+        <v>89</v>
+      </c>
+      <c r="J15">
+        <v>2026</v>
+      </c>
+      <c r="K15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="B16" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="D16" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E16" t="s">
+        <v>37</v>
+      </c>
+      <c r="F16" t="s">
+        <v>93</v>
+      </c>
+      <c r="G16" t="s">
+        <v>18</v>
+      </c>
+      <c r="H16" t="s">
+        <v>19</v>
+      </c>
+      <c r="I16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J16">
+        <v>2026</v>
+      </c>
+      <c r="K16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C17" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="D17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E17" t="s">
+        <v>37</v>
+      </c>
+      <c r="F17" t="s">
+        <v>98</v>
+      </c>
+      <c r="G17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H17" t="s">
+        <v>32</v>
+      </c>
+      <c r="I17" t="s">
+        <v>99</v>
+      </c>
+      <c r="J17">
+        <v>2026</v>
+      </c>
+      <c r="K17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="B18" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="D18" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E18" t="s">
+        <v>103</v>
+      </c>
+      <c r="F18" t="s">
+        <v>104</v>
+      </c>
+      <c r="G18" t="s">
+        <v>18</v>
+      </c>
+      <c r="H18" t="s">
+        <v>105</v>
+      </c>
+      <c r="I18" t="s">
+        <v>106</v>
+      </c>
+      <c r="J18">
+        <v>2025</v>
+      </c>
+      <c r="K18" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="B19" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="D19" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E19" t="s">
+        <v>110</v>
+      </c>
+      <c r="F19" t="s">
+        <v>111</v>
+      </c>
+      <c r="G19" t="s">
+        <v>31</v>
+      </c>
+      <c r="H19" t="s">
+        <v>32</v>
+      </c>
+      <c r="I19" t="s">
+        <v>112</v>
+      </c>
+      <c r="J19">
+        <v>2026</v>
+      </c>
+      <c r="K19" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="B20" t="s">
-        <v>94</v>
+        <v>115</v>
       </c>
       <c r="D20" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E20" t="s">
+        <v>110</v>
+      </c>
+      <c r="F20" t="s">
+        <v>116</v>
+      </c>
+      <c r="G20" t="s">
+        <v>31</v>
+      </c>
+      <c r="H20" t="s">
+        <v>117</v>
+      </c>
+      <c r="I20" t="s">
+        <v>118</v>
+      </c>
+      <c r="J20">
+        <v>2025</v>
+      </c>
+      <c r="K20" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="B21" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="D21" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E21" t="s">
+        <v>110</v>
+      </c>
+      <c r="F21" t="s">
+        <v>121</v>
+      </c>
+      <c r="G21" t="s">
+        <v>31</v>
+      </c>
+      <c r="H21" t="s">
+        <v>117</v>
+      </c>
+      <c r="I21" t="s">
+        <v>122</v>
+      </c>
+      <c r="J21">
+        <v>2025</v>
+      </c>
+      <c r="K21" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>97</v>
+        <v>123</v>
       </c>
       <c r="B22" t="s">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="C22" t="s">
-        <v>99</v>
+        <v>125</v>
       </c>
       <c r="D22" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E22" t="s">
+        <v>103</v>
+      </c>
+      <c r="F22" t="s">
+        <v>126</v>
+      </c>
+      <c r="G22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H22" t="s">
+        <v>127</v>
+      </c>
+      <c r="I22" t="s">
+        <v>128</v>
+      </c>
+      <c r="J22">
+        <v>2025</v>
+      </c>
+      <c r="K22" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="B23" t="s">
-        <v>101</v>
+        <v>130</v>
       </c>
       <c r="D23" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E23" t="s">
+        <v>110</v>
+      </c>
+      <c r="F23" t="s">
+        <v>131</v>
+      </c>
+      <c r="G23" t="s">
+        <v>51</v>
+      </c>
+      <c r="H23" t="s">
+        <v>117</v>
+      </c>
+      <c r="I23" t="s">
+        <v>132</v>
+      </c>
+      <c r="J23">
+        <v>2025</v>
+      </c>
+      <c r="K23" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>102</v>
+        <v>133</v>
       </c>
       <c r="B24" t="s">
-        <v>103</v>
+        <v>134</v>
       </c>
       <c r="C24" t="s">
-        <v>104</v>
+        <v>135</v>
       </c>
       <c r="D24" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E24" t="s">
+        <v>37</v>
+      </c>
+      <c r="F24" t="s">
+        <v>136</v>
+      </c>
+      <c r="G24" t="s">
+        <v>18</v>
+      </c>
+      <c r="H24" t="s">
+        <v>40</v>
+      </c>
+      <c r="I24" t="s">
+        <v>137</v>
+      </c>
+      <c r="J24">
+        <v>2026</v>
+      </c>
+      <c r="K24" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>105</v>
+        <v>138</v>
       </c>
       <c r="B25" t="s">
-        <v>106</v>
+        <v>139</v>
       </c>
       <c r="D25" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F25" t="s">
+        <v>140</v>
+      </c>
+      <c r="G25" t="s">
+        <v>31</v>
+      </c>
+      <c r="H25" t="s">
+        <v>32</v>
+      </c>
+      <c r="I25" t="s">
+        <v>141</v>
+      </c>
+      <c r="J25">
+        <v>2026</v>
+      </c>
+      <c r="K25" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>107</v>
+        <v>142</v>
       </c>
       <c r="B26" t="s">
-        <v>108</v>
+        <v>143</v>
       </c>
       <c r="C26" t="s">
-        <v>109</v>
+        <v>144</v>
       </c>
       <c r="D26" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E26" t="s">
+        <v>110</v>
+      </c>
+      <c r="F26" t="s">
+        <v>145</v>
+      </c>
+      <c r="G26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H26" t="s">
+        <v>40</v>
+      </c>
+      <c r="I26" t="s">
+        <v>146</v>
+      </c>
+      <c r="J26">
+        <v>2025</v>
+      </c>
+      <c r="K26" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>110</v>
+        <v>147</v>
       </c>
       <c r="B27" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
       <c r="C27" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
       <c r="D27" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E27" t="s">
+        <v>37</v>
+      </c>
+      <c r="F27" t="s">
+        <v>150</v>
+      </c>
+      <c r="G27" t="s">
+        <v>151</v>
+      </c>
+      <c r="H27" t="s">
+        <v>32</v>
+      </c>
+      <c r="I27" t="s">
+        <v>152</v>
+      </c>
+      <c r="J27">
+        <v>2026</v>
+      </c>
+      <c r="K27" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>113</v>
+        <v>153</v>
       </c>
       <c r="B28" t="s">
-        <v>114</v>
+        <v>154</v>
       </c>
       <c r="C28" t="s">
-        <v>115</v>
+        <v>155</v>
       </c>
       <c r="D28" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E28" t="s">
+        <v>110</v>
+      </c>
+      <c r="F28" t="s">
+        <v>156</v>
+      </c>
+      <c r="G28" t="s">
+        <v>18</v>
+      </c>
+      <c r="H28" t="s">
+        <v>19</v>
+      </c>
+      <c r="I28" t="s">
+        <v>157</v>
+      </c>
+      <c r="J28">
+        <v>2025</v>
+      </c>
+      <c r="K28" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>116</v>
+        <v>158</v>
       </c>
       <c r="B29" t="s">
-        <v>117</v>
+        <v>159</v>
       </c>
       <c r="C29" t="s">
-        <v>118</v>
+        <v>160</v>
       </c>
       <c r="D29" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E29" t="s">
+        <v>161</v>
+      </c>
+      <c r="F29" t="s">
+        <v>162</v>
+      </c>
+      <c r="G29" t="s">
+        <v>18</v>
+      </c>
+      <c r="H29" t="s">
+        <v>127</v>
+      </c>
+      <c r="I29" t="s">
+        <v>163</v>
+      </c>
+      <c r="J29">
+        <v>2023</v>
+      </c>
+      <c r="K29" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>119</v>
-      </c>
-      <c r="B30" t="s">
-        <v>120</v>
-      </c>
-      <c r="C30" t="s">
-        <v>121</v>
+        <v>165</v>
       </c>
       <c r="D30" t="s">
         <v>15</v>
+      </c>
+      <c r="E30" t="s">
+        <v>161</v>
+      </c>
+      <c r="F30" t="s">
+        <v>166</v>
+      </c>
+      <c r="G30" t="s">
+        <v>18</v>
+      </c>
+      <c r="H30" t="s">
+        <v>127</v>
+      </c>
+      <c r="I30" t="s">
+        <v>167</v>
+      </c>
+      <c r="J30">
+        <v>2023</v>
+      </c>
+      <c r="K30" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>168</v>
+      </c>
+      <c r="D31" t="s">
+        <v>29</v>
+      </c>
+      <c r="E31" t="s">
+        <v>161</v>
+      </c>
+      <c r="F31" t="s">
+        <v>169</v>
+      </c>
+      <c r="G31" t="s">
+        <v>31</v>
+      </c>
+      <c r="H31" t="s">
+        <v>32</v>
+      </c>
+      <c r="I31" t="s">
+        <v>170</v>
+      </c>
+      <c r="J31">
+        <v>2023</v>
+      </c>
+      <c r="K31" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>171</v>
+      </c>
+      <c r="D32" t="s">
+        <v>29</v>
+      </c>
+      <c r="E32" t="s">
+        <v>161</v>
+      </c>
+      <c r="F32" t="s">
+        <v>169</v>
+      </c>
+      <c r="G32" t="s">
+        <v>31</v>
+      </c>
+      <c r="H32" t="s">
+        <v>32</v>
+      </c>
+      <c r="I32" t="s">
+        <v>170</v>
+      </c>
+      <c r="J32">
+        <v>2023</v>
+      </c>
+      <c r="K32" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>172</v>
+      </c>
+      <c r="D33" t="s">
+        <v>15</v>
+      </c>
+      <c r="E33" t="s">
+        <v>173</v>
+      </c>
+      <c r="F33" t="s">
+        <v>174</v>
+      </c>
+      <c r="G33" t="s">
+        <v>31</v>
+      </c>
+      <c r="H33" t="s">
+        <v>105</v>
+      </c>
+      <c r="I33" t="s">
+        <v>175</v>
+      </c>
+      <c r="J33">
+        <v>2024</v>
+      </c>
+      <c r="K33" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Polish portfolio UX with glass Aero styling, bubble cursor, and video poster fixes
Add GSAP bubble cursor and shelve the liquid trail, deepen the Aero background, and apply glass-shell styling to the navbar, hero, and filters. Fix black video thumbnails with luminance-based poster extraction and hover preview poster overlays, plus intake chip and board refinements.
</commit_message>
<xml_diff>
--- a/content/portfolio-intake.xlsx
+++ b/content/portfolio-intake.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="178">
   <si>
     <t>source_file</t>
   </si>
@@ -527,6 +527,9 @@
   </si>
   <si>
     <t>kashef tbs.png</t>
+  </si>
+  <si>
+    <t>Infographic 2</t>
   </si>
   <si>
     <t>LTE Case.mp4</t>
@@ -1991,7 +1994,7 @@
         <v>161</v>
       </c>
       <c r="F32" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="G32" t="s">
         <v>31</v>
@@ -2011,16 +2014,16 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D33" t="s">
         <v>15</v>
       </c>
       <c r="E33" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G33" t="s">
         <v>31</v>
@@ -2029,13 +2032,13 @@
         <v>105</v>
       </c>
       <c r="I33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J33">
         <v>2024</v>
       </c>
       <c r="K33" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>